<commit_message>
Update EDB price data
</commit_message>
<xml_diff>
--- a/edb_data/DRAM合约平均价格.xlsx
+++ b/edb_data/DRAM合约平均价格.xlsx
@@ -4,12 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9060"/>
+    <workbookView windowWidth="27948" windowHeight="11700"/>
   </bookViews>
   <sheets>
     <sheet name="合约平均价_DRAM_DDR5(8Gb," sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1249,7 +1249,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1280,10 +1280,10 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="B3" s="4">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C3" s="4">
         <v>227</v>
@@ -1292,41 +1292,41 @@
         <v>119</v>
       </c>
       <c r="E3" s="4">
-        <v>33.5</v>
+        <v>40</v>
       </c>
       <c r="F3" s="4">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="B4" s="4">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C4" s="4">
-        <v>170</v>
+        <v>227</v>
       </c>
       <c r="D4" s="4">
-        <v>85</v>
+        <v>119</v>
       </c>
       <c r="E4" s="4">
-        <v>29.5</v>
+        <v>33.5</v>
       </c>
       <c r="F4" s="4">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3">
-        <v>46081</v>
+        <v>46112</v>
       </c>
       <c r="B5" s="4">
         <v>75</v>
       </c>
       <c r="C5" s="4">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D5" s="4">
         <v>85</v>
@@ -1340,107 +1340,107 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3">
-        <v>46053</v>
+        <v>46081</v>
       </c>
       <c r="B6" s="4">
         <v>75</v>
       </c>
       <c r="C6" s="4">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D6" s="4">
         <v>85</v>
       </c>
       <c r="E6" s="4">
-        <v>26</v>
+        <v>29.5</v>
       </c>
       <c r="F6" s="4">
-        <v>11.5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3">
-        <v>46022</v>
+        <v>46053</v>
       </c>
       <c r="B7" s="4">
-        <v>39.5</v>
+        <v>75</v>
       </c>
       <c r="C7" s="4">
-        <v>87</v>
+        <v>160</v>
       </c>
       <c r="D7" s="4">
-        <v>46.5</v>
+        <v>85</v>
       </c>
       <c r="E7" s="4">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F7" s="4">
-        <v>9.3</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3">
-        <v>45991</v>
+        <v>46022</v>
       </c>
       <c r="B8" s="4">
-        <v>36.5</v>
+        <v>39.5</v>
       </c>
       <c r="C8" s="4">
-        <v>73.5</v>
+        <v>87</v>
       </c>
       <c r="D8" s="4">
-        <v>39</v>
+        <v>46.5</v>
       </c>
       <c r="E8" s="4">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F8" s="4">
-        <v>8.1</v>
+        <v>9.3</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3">
-        <v>45961</v>
+        <v>45991</v>
       </c>
       <c r="B9" s="4">
-        <v>33.5</v>
+        <v>36.5</v>
       </c>
       <c r="C9" s="4">
-        <v>60</v>
+        <v>73.5</v>
       </c>
       <c r="D9" s="4">
-        <v>31.5</v>
+        <v>39</v>
       </c>
       <c r="E9" s="4">
-        <v>14.8</v>
+        <v>18</v>
       </c>
       <c r="F9" s="4">
-        <v>7</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3">
-        <v>45930</v>
+        <v>45961</v>
       </c>
       <c r="B10" s="4">
-        <v>26.75</v>
+        <v>33.5</v>
       </c>
       <c r="C10" s="4">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D10" s="4">
-        <v>27</v>
+        <v>31.5</v>
       </c>
       <c r="E10" s="4">
-        <v>13.2</v>
+        <v>14.8</v>
       </c>
       <c r="F10" s="4">
-        <v>6.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3">
-        <v>45900</v>
+        <v>45930</v>
       </c>
       <c r="B11" s="4">
         <v>26.75</v>
@@ -1452,55 +1452,55 @@
         <v>27</v>
       </c>
       <c r="E11" s="4">
-        <v>12</v>
+        <v>13.2</v>
       </c>
       <c r="F11" s="4">
-        <v>5.7</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3">
-        <v>45869</v>
+        <v>45900</v>
       </c>
       <c r="B12" s="4">
-        <v>25.5</v>
+        <v>26.75</v>
       </c>
       <c r="C12" s="4">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" s="4">
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="E12" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F12" s="4">
-        <v>3.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="3">
-        <v>45838</v>
+        <v>45869</v>
       </c>
       <c r="B13" s="4">
-        <v>24.5</v>
+        <v>25.5</v>
       </c>
       <c r="C13" s="4">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D13" s="4">
-        <v>19.5</v>
+        <v>26.5</v>
       </c>
       <c r="E13" s="4">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="F13" s="4">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="3">
-        <v>45808</v>
+        <v>45838</v>
       </c>
       <c r="B14" s="4">
         <v>24.5</v>
@@ -1512,55 +1512,55 @@
         <v>19.5</v>
       </c>
       <c r="E14" s="4">
-        <v>3.6</v>
+        <v>5.5</v>
       </c>
       <c r="F14" s="4">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="3">
-        <v>45777</v>
+        <v>45808</v>
       </c>
       <c r="B15" s="4">
         <v>24.5</v>
       </c>
       <c r="C15" s="4">
-        <v>33.5</v>
+        <v>38</v>
       </c>
       <c r="D15" s="4">
-        <v>17.25</v>
+        <v>19.5</v>
       </c>
       <c r="E15" s="4">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="F15" s="4">
-        <v>1.65</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="3">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="B16" s="4">
-        <v>23</v>
+        <v>24.5</v>
       </c>
       <c r="C16" s="4">
-        <v>32</v>
+        <v>33.5</v>
       </c>
       <c r="D16" s="4">
-        <v>16.5</v>
+        <v>17.25</v>
       </c>
       <c r="E16" s="4">
-        <v>2.55</v>
+        <v>3.2</v>
       </c>
       <c r="F16" s="4">
-        <v>1.35</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3">
-        <v>45716</v>
+        <v>45747</v>
       </c>
       <c r="B17" s="4">
         <v>23</v>
@@ -1580,10 +1580,10 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3">
-        <v>45688</v>
+        <v>45716</v>
       </c>
       <c r="B18" s="4">
-        <v>23.5</v>
+        <v>23</v>
       </c>
       <c r="C18" s="4">
         <v>32</v>
@@ -1600,27 +1600,27 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="3">
-        <v>45657</v>
+        <v>45688</v>
       </c>
       <c r="B19" s="4">
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="C19" s="4">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D19" s="4">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="E19" s="4">
         <v>2.55</v>
       </c>
       <c r="F19" s="4">
-        <v>0</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="3">
-        <v>45626</v>
+        <v>45657</v>
       </c>
       <c r="B20" s="4">
         <v>25.5</v>
@@ -1640,19 +1640,19 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3">
-        <v>45596</v>
+        <v>45626</v>
       </c>
       <c r="B21" s="4">
-        <v>27</v>
+        <v>25.5</v>
       </c>
       <c r="C21" s="4">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D21" s="4">
-        <v>21</v>
+        <v>18.5</v>
       </c>
       <c r="E21" s="4">
-        <v>3.2</v>
+        <v>2.55</v>
       </c>
       <c r="F21" s="4">
         <v>0</v>
@@ -1660,7 +1660,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3">
-        <v>45565</v>
+        <v>45596</v>
       </c>
       <c r="B22" s="4">
         <v>27</v>
@@ -1675,12 +1675,12 @@
         <v>3.2</v>
       </c>
       <c r="F22" s="4">
-        <v>1.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3">
-        <v>45535</v>
+        <v>45565</v>
       </c>
       <c r="B23" s="4">
         <v>27</v>
@@ -1692,15 +1692,15 @@
         <v>21</v>
       </c>
       <c r="E23" s="4">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="F23" s="4">
-        <v>2.05</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="3">
-        <v>45504</v>
+        <v>45535</v>
       </c>
       <c r="B24" s="4">
         <v>27</v>
@@ -1712,24 +1712,24 @@
         <v>21</v>
       </c>
       <c r="E24" s="4">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="F24" s="4">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="3">
-        <v>45473</v>
+        <v>45504</v>
       </c>
       <c r="B25" s="4">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C25" s="4">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D25" s="4">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E25" s="4">
         <v>4.2</v>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="3">
-        <v>45443</v>
+        <v>45473</v>
       </c>
       <c r="B26" s="4">
         <v>24</v>
@@ -1760,7 +1760,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="3">
-        <v>45412</v>
+        <v>45443</v>
       </c>
       <c r="B27" s="4">
         <v>24</v>
@@ -1780,27 +1780,27 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="3">
-        <v>45382</v>
+        <v>45412</v>
       </c>
       <c r="B28" s="4">
-        <v>20.5</v>
+        <v>24</v>
       </c>
       <c r="C28" s="4">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D28" s="4">
-        <v>16.5</v>
+        <v>19</v>
       </c>
       <c r="E28" s="4">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
       <c r="F28" s="4">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="3">
-        <v>45351</v>
+        <v>45382</v>
       </c>
       <c r="B29" s="4">
         <v>20.5</v>
@@ -1820,7 +1820,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="3">
-        <v>45322</v>
+        <v>45351</v>
       </c>
       <c r="B30" s="4">
         <v>20.5</v>
@@ -1840,27 +1840,27 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="3">
-        <v>45291</v>
+        <v>45322</v>
       </c>
       <c r="B31" s="4">
-        <v>17.5</v>
+        <v>20.5</v>
       </c>
       <c r="C31" s="4">
-        <v>26.4</v>
+        <v>32</v>
       </c>
       <c r="D31" s="4">
-        <v>13.7</v>
+        <v>16.5</v>
       </c>
       <c r="E31" s="4">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="F31" s="4">
-        <v>1.65</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="3">
-        <v>45260</v>
+        <v>45291</v>
       </c>
       <c r="B32" s="4">
         <v>17.5</v>
@@ -1872,18 +1872,18 @@
         <v>13.7</v>
       </c>
       <c r="E32" s="4">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="F32" s="4">
-        <v>1.55</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="3">
-        <v>45230</v>
+        <v>45260</v>
       </c>
       <c r="B33" s="4">
-        <v>17</v>
+        <v>17.5</v>
       </c>
       <c r="C33" s="4">
         <v>26.4</v>
@@ -1892,35 +1892,35 @@
         <v>13.7</v>
       </c>
       <c r="E33" s="4">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="F33" s="4">
-        <v>1.5</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="3">
-        <v>45199</v>
+        <v>45230</v>
       </c>
       <c r="B34" s="4">
-        <v>15.3</v>
+        <v>17</v>
       </c>
       <c r="C34" s="4">
-        <v>23.8</v>
+        <v>26.4</v>
       </c>
       <c r="D34" s="4">
-        <v>12.4</v>
+        <v>13.7</v>
       </c>
       <c r="E34" s="4">
-        <v>2.73</v>
+        <v>3</v>
       </c>
       <c r="F34" s="4">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="3">
-        <v>45169</v>
+        <v>45199</v>
       </c>
       <c r="B35" s="4">
         <v>15.3</v>
@@ -1940,101 +1940,121 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3">
-        <v>45138</v>
+        <v>45169</v>
       </c>
       <c r="B36" s="4">
         <v>15.3</v>
       </c>
       <c r="C36" s="4">
-        <v>24.4</v>
+        <v>23.8</v>
       </c>
       <c r="D36" s="4">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="E36" s="4">
-        <v>2.8</v>
+        <v>2.73</v>
       </c>
       <c r="F36" s="4">
-        <v>1.34</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="3">
-        <v>45107</v>
+        <v>45138</v>
       </c>
       <c r="B37" s="4">
-        <v>14.835</v>
+        <v>15.3</v>
       </c>
       <c r="C37" s="4">
-        <v>24.8</v>
+        <v>24.4</v>
       </c>
       <c r="D37" s="4">
-        <v>12.9</v>
+        <v>12.7</v>
       </c>
       <c r="E37" s="4">
-        <v>2.85</v>
+        <v>2.8</v>
       </c>
       <c r="F37" s="4">
-        <v>1.36</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="3">
-        <v>45077</v>
+        <v>45107</v>
       </c>
       <c r="B38" s="4">
-        <v>15.18</v>
+        <v>14.835</v>
       </c>
       <c r="C38" s="4">
-        <v>25.4</v>
+        <v>24.8</v>
       </c>
       <c r="D38" s="4">
-        <v>13.2</v>
+        <v>12.9</v>
       </c>
       <c r="E38" s="4">
-        <v>2.93</v>
+        <v>2.85</v>
       </c>
       <c r="F38" s="4">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="3">
-        <v>45046</v>
+        <v>45077</v>
       </c>
       <c r="B39" s="4">
-        <v>15.64</v>
+        <v>15.18</v>
       </c>
       <c r="C39" s="4">
-        <v>26.2</v>
+        <v>25.4</v>
       </c>
       <c r="D39" s="4">
-        <v>13.6</v>
+        <v>13.2</v>
       </c>
       <c r="E39" s="4">
-        <v>3.03</v>
+        <v>2.93</v>
       </c>
       <c r="F39" s="4">
-        <v>1.45</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="3">
+        <v>45046</v>
+      </c>
+      <c r="B40" s="4">
+        <v>15.64</v>
+      </c>
+      <c r="C40" s="4">
+        <v>26.2</v>
+      </c>
+      <c r="D40" s="4">
+        <v>13.6</v>
+      </c>
+      <c r="E40" s="4">
+        <v>3.03</v>
+      </c>
+      <c r="F40" s="4">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="3">
         <v>45016</v>
       </c>
-      <c r="B40" s="4">
+      <c r="B41" s="4">
         <v>18.975</v>
       </c>
-      <c r="C40" s="4">
+      <c r="C41" s="4">
         <v>32</v>
       </c>
-      <c r="D40" s="4">
+      <c r="D41" s="4">
         <v>16.5</v>
       </c>
-      <c r="E40" s="4">
+      <c r="E41" s="4">
         <v>3.75</v>
       </c>
-      <c r="F40" s="4">
+      <c r="F41" s="4">
         <v>1.81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update EDB prices and remove duplicate report summary
</commit_message>
<xml_diff>
--- a/edb_data/DRAM合约平均价格.xlsx
+++ b/edb_data/DRAM合约平均价格.xlsx
@@ -4,12 +4,15 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="12300"/>
+    <workbookView windowWidth="22188" windowHeight="8460"/>
   </bookViews>
   <sheets>
     <sheet name="合约平均价_DRAM_DDR5(8Gb," sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" calcMode="manual"/>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -991,6 +994,26 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+      <sheetName val="Sheet2"/>
+      <sheetName val="Sheet3"/>
+    </sheetNames>
+    <definedNames>
+      <definedName name="edb"/>
+    </definedNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -1254,7 +1277,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="str">
-        <f>edb()</f>
+        <f>[1]!edb()</f>
         <v>Wind</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update EDB prices for August 3
</commit_message>
<xml_diff>
--- a/edb_data/DRAM合约平均价格.xlsx
+++ b/edb_data/DRAM合约平均价格.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="12300"/>
+    <workbookView windowWidth="22188" windowHeight="9060"/>
   </bookViews>
   <sheets>
     <sheet name="合约平均价_DRAM_DDR5(8Gb," sheetId="1" r:id="rId1"/>
@@ -705,13 +705,19 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1272,7 +1278,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1303,10 +1309,10 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3">
-        <v>46173</v>
+        <v>46203</v>
       </c>
       <c r="B3" s="4">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C3" s="4">
         <v>227</v>
@@ -1315,18 +1321,18 @@
         <v>119</v>
       </c>
       <c r="E3" s="4">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F3" s="4">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="B4" s="4">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" s="4">
         <v>227</v>
@@ -1335,41 +1341,41 @@
         <v>119</v>
       </c>
       <c r="E4" s="4">
-        <v>33.5</v>
+        <v>40</v>
       </c>
       <c r="F4" s="4">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="B5" s="4">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C5" s="4">
-        <v>170</v>
+        <v>227</v>
       </c>
       <c r="D5" s="4">
-        <v>85</v>
+        <v>119</v>
       </c>
       <c r="E5" s="4">
-        <v>29.5</v>
+        <v>33.5</v>
       </c>
       <c r="F5" s="4">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3">
-        <v>46081</v>
+        <v>46112</v>
       </c>
       <c r="B6" s="4">
         <v>75</v>
       </c>
       <c r="C6" s="4">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D6" s="4">
         <v>85</v>
@@ -1383,107 +1389,107 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3">
-        <v>46053</v>
+        <v>46081</v>
       </c>
       <c r="B7" s="4">
         <v>75</v>
       </c>
       <c r="C7" s="4">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D7" s="4">
         <v>85</v>
       </c>
       <c r="E7" s="4">
-        <v>26</v>
+        <v>29.5</v>
       </c>
       <c r="F7" s="4">
-        <v>11.5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3">
-        <v>46022</v>
+        <v>46053</v>
       </c>
       <c r="B8" s="4">
-        <v>39.5</v>
+        <v>75</v>
       </c>
       <c r="C8" s="4">
-        <v>87</v>
+        <v>160</v>
       </c>
       <c r="D8" s="4">
-        <v>46.5</v>
+        <v>85</v>
       </c>
       <c r="E8" s="4">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F8" s="4">
-        <v>9.3</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3">
-        <v>45991</v>
+        <v>46022</v>
       </c>
       <c r="B9" s="4">
-        <v>36.5</v>
+        <v>39.5</v>
       </c>
       <c r="C9" s="4">
-        <v>73.5</v>
+        <v>87</v>
       </c>
       <c r="D9" s="4">
-        <v>39</v>
+        <v>46.5</v>
       </c>
       <c r="E9" s="4">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F9" s="4">
-        <v>8.1</v>
+        <v>9.3</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3">
-        <v>45961</v>
+        <v>45991</v>
       </c>
       <c r="B10" s="4">
-        <v>33.5</v>
+        <v>36.5</v>
       </c>
       <c r="C10" s="4">
-        <v>60</v>
+        <v>73.5</v>
       </c>
       <c r="D10" s="4">
-        <v>31.5</v>
+        <v>39</v>
       </c>
       <c r="E10" s="4">
-        <v>14.8</v>
+        <v>18</v>
       </c>
       <c r="F10" s="4">
-        <v>7</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3">
-        <v>45930</v>
+        <v>45961</v>
       </c>
       <c r="B11" s="4">
-        <v>26.75</v>
+        <v>33.5</v>
       </c>
       <c r="C11" s="4">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D11" s="4">
-        <v>27</v>
+        <v>31.5</v>
       </c>
       <c r="E11" s="4">
-        <v>13.2</v>
+        <v>14.8</v>
       </c>
       <c r="F11" s="4">
-        <v>6.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3">
-        <v>45900</v>
+        <v>45930</v>
       </c>
       <c r="B12" s="4">
         <v>26.75</v>
@@ -1495,55 +1501,55 @@
         <v>27</v>
       </c>
       <c r="E12" s="4">
-        <v>12</v>
+        <v>13.2</v>
       </c>
       <c r="F12" s="4">
-        <v>5.7</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="3">
-        <v>45869</v>
+        <v>45900</v>
       </c>
       <c r="B13" s="4">
-        <v>25.5</v>
+        <v>26.75</v>
       </c>
       <c r="C13" s="4">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D13" s="4">
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="E13" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F13" s="4">
-        <v>3.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="3">
-        <v>45838</v>
+        <v>45869</v>
       </c>
       <c r="B14" s="4">
-        <v>24.5</v>
+        <v>25.5</v>
       </c>
       <c r="C14" s="4">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D14" s="4">
-        <v>19.5</v>
+        <v>26.5</v>
       </c>
       <c r="E14" s="4">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="F14" s="4">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="3">
-        <v>45808</v>
+        <v>45838</v>
       </c>
       <c r="B15" s="4">
         <v>24.5</v>
@@ -1555,55 +1561,55 @@
         <v>19.5</v>
       </c>
       <c r="E15" s="4">
-        <v>3.6</v>
+        <v>5.5</v>
       </c>
       <c r="F15" s="4">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="3">
-        <v>45777</v>
+        <v>45808</v>
       </c>
       <c r="B16" s="4">
         <v>24.5</v>
       </c>
       <c r="C16" s="4">
-        <v>33.5</v>
+        <v>38</v>
       </c>
       <c r="D16" s="4">
-        <v>17.25</v>
+        <v>19.5</v>
       </c>
       <c r="E16" s="4">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="F16" s="4">
-        <v>1.65</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="B17" s="4">
-        <v>23</v>
+        <v>24.5</v>
       </c>
       <c r="C17" s="4">
-        <v>32</v>
+        <v>33.5</v>
       </c>
       <c r="D17" s="4">
-        <v>16.5</v>
+        <v>17.25</v>
       </c>
       <c r="E17" s="4">
-        <v>2.55</v>
+        <v>3.2</v>
       </c>
       <c r="F17" s="4">
-        <v>1.35</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3">
-        <v>45716</v>
+        <v>45747</v>
       </c>
       <c r="B18" s="4">
         <v>23</v>
@@ -1623,10 +1629,10 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="3">
-        <v>45688</v>
+        <v>45716</v>
       </c>
       <c r="B19" s="4">
-        <v>23.5</v>
+        <v>23</v>
       </c>
       <c r="C19" s="4">
         <v>32</v>
@@ -1643,27 +1649,27 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="3">
-        <v>45657</v>
+        <v>45688</v>
       </c>
       <c r="B20" s="4">
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="C20" s="4">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D20" s="4">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="E20" s="4">
         <v>2.55</v>
       </c>
       <c r="F20" s="4">
-        <v>0</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3">
-        <v>45626</v>
+        <v>45657</v>
       </c>
       <c r="B21" s="4">
         <v>25.5</v>
@@ -1683,19 +1689,19 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3">
-        <v>45596</v>
+        <v>45626</v>
       </c>
       <c r="B22" s="4">
-        <v>27</v>
+        <v>25.5</v>
       </c>
       <c r="C22" s="4">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D22" s="4">
-        <v>21</v>
+        <v>18.5</v>
       </c>
       <c r="E22" s="4">
-        <v>3.2</v>
+        <v>2.55</v>
       </c>
       <c r="F22" s="4">
         <v>0</v>
@@ -1703,7 +1709,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3">
-        <v>45565</v>
+        <v>45596</v>
       </c>
       <c r="B23" s="4">
         <v>27</v>
@@ -1718,12 +1724,12 @@
         <v>3.2</v>
       </c>
       <c r="F23" s="4">
-        <v>1.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="3">
-        <v>45535</v>
+        <v>45565</v>
       </c>
       <c r="B24" s="4">
         <v>27</v>
@@ -1735,15 +1741,15 @@
         <v>21</v>
       </c>
       <c r="E24" s="4">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="F24" s="4">
-        <v>2.05</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="3">
-        <v>45504</v>
+        <v>45535</v>
       </c>
       <c r="B25" s="4">
         <v>27</v>
@@ -1755,24 +1761,24 @@
         <v>21</v>
       </c>
       <c r="E25" s="4">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="F25" s="4">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="3">
-        <v>45473</v>
+        <v>45504</v>
       </c>
       <c r="B26" s="4">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C26" s="4">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D26" s="4">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E26" s="4">
         <v>4.2</v>
@@ -1783,7 +1789,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="3">
-        <v>45443</v>
+        <v>45473</v>
       </c>
       <c r="B27" s="4">
         <v>24</v>
@@ -1803,7 +1809,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="3">
-        <v>45412</v>
+        <v>45443</v>
       </c>
       <c r="B28" s="4">
         <v>24</v>
@@ -1823,27 +1829,27 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="3">
-        <v>45382</v>
+        <v>45412</v>
       </c>
       <c r="B29" s="4">
-        <v>20.5</v>
+        <v>24</v>
       </c>
       <c r="C29" s="4">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D29" s="4">
-        <v>16.5</v>
+        <v>19</v>
       </c>
       <c r="E29" s="4">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
       <c r="F29" s="4">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="3">
-        <v>45351</v>
+        <v>45382</v>
       </c>
       <c r="B30" s="4">
         <v>20.5</v>
@@ -1863,7 +1869,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="3">
-        <v>45322</v>
+        <v>45351</v>
       </c>
       <c r="B31" s="4">
         <v>20.5</v>
@@ -1883,27 +1889,27 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="3">
-        <v>45291</v>
+        <v>45322</v>
       </c>
       <c r="B32" s="4">
-        <v>17.5</v>
+        <v>20.5</v>
       </c>
       <c r="C32" s="4">
-        <v>26.4</v>
+        <v>32</v>
       </c>
       <c r="D32" s="4">
-        <v>13.7</v>
+        <v>16.5</v>
       </c>
       <c r="E32" s="4">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="F32" s="4">
-        <v>1.65</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="3">
-        <v>45260</v>
+        <v>45291</v>
       </c>
       <c r="B33" s="4">
         <v>17.5</v>
@@ -1915,18 +1921,18 @@
         <v>13.7</v>
       </c>
       <c r="E33" s="4">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="F33" s="4">
-        <v>1.55</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="3">
-        <v>45230</v>
+        <v>45260</v>
       </c>
       <c r="B34" s="4">
-        <v>17</v>
+        <v>17.5</v>
       </c>
       <c r="C34" s="4">
         <v>26.4</v>
@@ -1935,35 +1941,35 @@
         <v>13.7</v>
       </c>
       <c r="E34" s="4">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="F34" s="4">
-        <v>1.5</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="3">
-        <v>45199</v>
+        <v>45230</v>
       </c>
       <c r="B35" s="4">
-        <v>15.3</v>
+        <v>17</v>
       </c>
       <c r="C35" s="4">
-        <v>23.8</v>
+        <v>26.4</v>
       </c>
       <c r="D35" s="4">
-        <v>12.4</v>
+        <v>13.7</v>
       </c>
       <c r="E35" s="4">
-        <v>2.73</v>
+        <v>3</v>
       </c>
       <c r="F35" s="4">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3">
-        <v>45169</v>
+        <v>45199</v>
       </c>
       <c r="B36" s="4">
         <v>15.3</v>
@@ -1983,101 +1989,121 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="3">
-        <v>45138</v>
+        <v>45169</v>
       </c>
       <c r="B37" s="4">
         <v>15.3</v>
       </c>
       <c r="C37" s="4">
-        <v>24.4</v>
+        <v>23.8</v>
       </c>
       <c r="D37" s="4">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="E37" s="4">
-        <v>2.8</v>
+        <v>2.73</v>
       </c>
       <c r="F37" s="4">
-        <v>1.34</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="3">
-        <v>45107</v>
+        <v>45138</v>
       </c>
       <c r="B38" s="4">
-        <v>14.835</v>
+        <v>15.3</v>
       </c>
       <c r="C38" s="4">
-        <v>24.8</v>
+        <v>24.4</v>
       </c>
       <c r="D38" s="4">
-        <v>12.9</v>
+        <v>12.7</v>
       </c>
       <c r="E38" s="4">
-        <v>2.85</v>
+        <v>2.8</v>
       </c>
       <c r="F38" s="4">
-        <v>1.36</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="3">
-        <v>45077</v>
+        <v>45107</v>
       </c>
       <c r="B39" s="4">
-        <v>15.18</v>
+        <v>14.835</v>
       </c>
       <c r="C39" s="4">
-        <v>25.4</v>
+        <v>24.8</v>
       </c>
       <c r="D39" s="4">
-        <v>13.2</v>
+        <v>12.9</v>
       </c>
       <c r="E39" s="4">
-        <v>2.93</v>
+        <v>2.85</v>
       </c>
       <c r="F39" s="4">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="3">
-        <v>45046</v>
+        <v>45077</v>
       </c>
       <c r="B40" s="4">
-        <v>15.64</v>
+        <v>15.18</v>
       </c>
       <c r="C40" s="4">
-        <v>26.2</v>
+        <v>25.4</v>
       </c>
       <c r="D40" s="4">
-        <v>13.6</v>
+        <v>13.2</v>
       </c>
       <c r="E40" s="4">
-        <v>3.03</v>
+        <v>2.93</v>
       </c>
       <c r="F40" s="4">
-        <v>1.45</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="3">
+        <v>45046</v>
+      </c>
+      <c r="B41" s="4">
+        <v>15.64</v>
+      </c>
+      <c r="C41" s="4">
+        <v>26.2</v>
+      </c>
+      <c r="D41" s="4">
+        <v>13.6</v>
+      </c>
+      <c r="E41" s="4">
+        <v>3.03</v>
+      </c>
+      <c r="F41" s="4">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="5">
         <v>45016</v>
       </c>
-      <c r="B41" s="4">
+      <c r="B42" s="6">
         <v>18.975</v>
       </c>
-      <c r="C41" s="4">
+      <c r="C42" s="6">
         <v>32</v>
       </c>
-      <c r="D41" s="4">
+      <c r="D42" s="6">
         <v>16.5</v>
       </c>
-      <c r="E41" s="4">
+      <c r="E42" s="6">
         <v>3.75</v>
       </c>
-      <c r="F41" s="4">
+      <c r="F42" s="6">
         <v>1.81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update EDB prices for August 10
</commit_message>
<xml_diff>
--- a/edb_data/DRAM合约平均价格.xlsx
+++ b/edb_data/DRAM合约平均价格.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9060"/>
+    <workbookView windowWidth="27948" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="合约平均价_DRAM_DDR5(8Gb," sheetId="1" r:id="rId1"/>
@@ -705,19 +705,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -2088,22 +2082,22 @@
       </c>
     </row>
     <row r="42" spans="1:6">
-      <c r="A42" s="5">
+      <c r="A42" s="3">
         <v>45016</v>
       </c>
-      <c r="B42" s="6">
+      <c r="B42" s="4">
         <v>18.975</v>
       </c>
-      <c r="C42" s="6">
+      <c r="C42" s="4">
         <v>32</v>
       </c>
-      <c r="D42" s="6">
+      <c r="D42" s="4">
         <v>16.5</v>
       </c>
-      <c r="E42" s="6">
+      <c r="E42" s="4">
         <v>3.75</v>
       </c>
-      <c r="F42" s="6">
+      <c r="F42" s="4">
         <v>1.81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update EDB prices for September 1
</commit_message>
<xml_diff>
--- a/edb_data/DRAM合约平均价格.xlsx
+++ b/edb_data/DRAM合约平均价格.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Codex\存储行业可视化看板网站制作\edb_data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="12300"/>
+    <workbookView windowWidth="24048" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="合约平均价_DRAM_DDR5(8Gb," sheetId="1" r:id="rId1"/>
@@ -705,13 +710,19 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1272,7 +1283,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1303,30 +1314,30 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="B3" s="4">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="C3" s="4">
-        <v>227</v>
+        <v>265</v>
       </c>
       <c r="D3" s="4">
-        <v>119</v>
+        <v>139</v>
       </c>
       <c r="E3" s="4">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F3" s="4">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3">
-        <v>46173</v>
+        <v>46203</v>
       </c>
       <c r="B4" s="4">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C4" s="4">
         <v>227</v>
@@ -1335,18 +1346,18 @@
         <v>119</v>
       </c>
       <c r="E4" s="4">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F4" s="4">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="B5" s="4">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C5" s="4">
         <v>227</v>
@@ -1355,41 +1366,41 @@
         <v>119</v>
       </c>
       <c r="E5" s="4">
-        <v>33.5</v>
+        <v>40</v>
       </c>
       <c r="F5" s="4">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="B6" s="4">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C6" s="4">
-        <v>170</v>
+        <v>227</v>
       </c>
       <c r="D6" s="4">
-        <v>85</v>
+        <v>119</v>
       </c>
       <c r="E6" s="4">
-        <v>29.5</v>
+        <v>33.5</v>
       </c>
       <c r="F6" s="4">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3">
-        <v>46081</v>
+        <v>46112</v>
       </c>
       <c r="B7" s="4">
         <v>75</v>
       </c>
       <c r="C7" s="4">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D7" s="4">
         <v>85</v>
@@ -1403,107 +1414,107 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3">
-        <v>46053</v>
+        <v>46081</v>
       </c>
       <c r="B8" s="4">
         <v>75</v>
       </c>
       <c r="C8" s="4">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D8" s="4">
         <v>85</v>
       </c>
       <c r="E8" s="4">
-        <v>26</v>
+        <v>29.5</v>
       </c>
       <c r="F8" s="4">
-        <v>11.5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3">
-        <v>46022</v>
+        <v>46053</v>
       </c>
       <c r="B9" s="4">
-        <v>39.5</v>
+        <v>75</v>
       </c>
       <c r="C9" s="4">
-        <v>87</v>
+        <v>160</v>
       </c>
       <c r="D9" s="4">
-        <v>46.5</v>
+        <v>85</v>
       </c>
       <c r="E9" s="4">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F9" s="4">
-        <v>9.3</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3">
-        <v>45991</v>
+        <v>46022</v>
       </c>
       <c r="B10" s="4">
-        <v>36.5</v>
+        <v>39.5</v>
       </c>
       <c r="C10" s="4">
-        <v>73.5</v>
+        <v>87</v>
       </c>
       <c r="D10" s="4">
-        <v>39</v>
+        <v>46.5</v>
       </c>
       <c r="E10" s="4">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F10" s="4">
-        <v>8.1</v>
+        <v>9.3</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3">
-        <v>45961</v>
+        <v>45991</v>
       </c>
       <c r="B11" s="4">
-        <v>33.5</v>
+        <v>36.5</v>
       </c>
       <c r="C11" s="4">
-        <v>60</v>
+        <v>73.5</v>
       </c>
       <c r="D11" s="4">
-        <v>31.5</v>
+        <v>39</v>
       </c>
       <c r="E11" s="4">
-        <v>14.8</v>
+        <v>18</v>
       </c>
       <c r="F11" s="4">
-        <v>7</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3">
-        <v>45930</v>
+        <v>45961</v>
       </c>
       <c r="B12" s="4">
-        <v>26.75</v>
+        <v>33.5</v>
       </c>
       <c r="C12" s="4">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D12" s="4">
-        <v>27</v>
+        <v>31.5</v>
       </c>
       <c r="E12" s="4">
-        <v>13.2</v>
+        <v>14.8</v>
       </c>
       <c r="F12" s="4">
-        <v>6.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="3">
-        <v>45900</v>
+        <v>45930</v>
       </c>
       <c r="B13" s="4">
         <v>26.75</v>
@@ -1515,55 +1526,55 @@
         <v>27</v>
       </c>
       <c r="E13" s="4">
-        <v>12</v>
+        <v>13.2</v>
       </c>
       <c r="F13" s="4">
-        <v>5.7</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="3">
-        <v>45869</v>
+        <v>45900</v>
       </c>
       <c r="B14" s="4">
-        <v>25.5</v>
+        <v>26.75</v>
       </c>
       <c r="C14" s="4">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D14" s="4">
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="E14" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F14" s="4">
-        <v>3.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="3">
-        <v>45838</v>
+        <v>45869</v>
       </c>
       <c r="B15" s="4">
-        <v>24.5</v>
+        <v>25.5</v>
       </c>
       <c r="C15" s="4">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D15" s="4">
-        <v>19.5</v>
+        <v>26.5</v>
       </c>
       <c r="E15" s="4">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="F15" s="4">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="3">
-        <v>45808</v>
+        <v>45838</v>
       </c>
       <c r="B16" s="4">
         <v>24.5</v>
@@ -1575,55 +1586,55 @@
         <v>19.5</v>
       </c>
       <c r="E16" s="4">
-        <v>3.6</v>
+        <v>5.5</v>
       </c>
       <c r="F16" s="4">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3">
-        <v>45777</v>
+        <v>45808</v>
       </c>
       <c r="B17" s="4">
         <v>24.5</v>
       </c>
       <c r="C17" s="4">
-        <v>33.5</v>
+        <v>38</v>
       </c>
       <c r="D17" s="4">
-        <v>17.25</v>
+        <v>19.5</v>
       </c>
       <c r="E17" s="4">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="F17" s="4">
-        <v>1.65</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="B18" s="4">
-        <v>23</v>
+        <v>24.5</v>
       </c>
       <c r="C18" s="4">
-        <v>32</v>
+        <v>33.5</v>
       </c>
       <c r="D18" s="4">
-        <v>16.5</v>
+        <v>17.25</v>
       </c>
       <c r="E18" s="4">
-        <v>2.55</v>
+        <v>3.2</v>
       </c>
       <c r="F18" s="4">
-        <v>1.35</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="3">
-        <v>45716</v>
+        <v>45747</v>
       </c>
       <c r="B19" s="4">
         <v>23</v>
@@ -1643,10 +1654,10 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="3">
-        <v>45688</v>
+        <v>45716</v>
       </c>
       <c r="B20" s="4">
-        <v>23.5</v>
+        <v>23</v>
       </c>
       <c r="C20" s="4">
         <v>32</v>
@@ -1663,27 +1674,27 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3">
-        <v>45657</v>
+        <v>45688</v>
       </c>
       <c r="B21" s="4">
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="C21" s="4">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D21" s="4">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="E21" s="4">
         <v>2.55</v>
       </c>
       <c r="F21" s="4">
-        <v>0</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3">
-        <v>45626</v>
+        <v>45657</v>
       </c>
       <c r="B22" s="4">
         <v>25.5</v>
@@ -1703,19 +1714,19 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3">
-        <v>45596</v>
+        <v>45626</v>
       </c>
       <c r="B23" s="4">
-        <v>27</v>
+        <v>25.5</v>
       </c>
       <c r="C23" s="4">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D23" s="4">
-        <v>21</v>
+        <v>18.5</v>
       </c>
       <c r="E23" s="4">
-        <v>3.2</v>
+        <v>2.55</v>
       </c>
       <c r="F23" s="4">
         <v>0</v>
@@ -1723,7 +1734,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="3">
-        <v>45565</v>
+        <v>45596</v>
       </c>
       <c r="B24" s="4">
         <v>27</v>
@@ -1738,12 +1749,12 @@
         <v>3.2</v>
       </c>
       <c r="F24" s="4">
-        <v>1.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="3">
-        <v>45535</v>
+        <v>45565</v>
       </c>
       <c r="B25" s="4">
         <v>27</v>
@@ -1755,15 +1766,15 @@
         <v>21</v>
       </c>
       <c r="E25" s="4">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="F25" s="4">
-        <v>2.05</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="3">
-        <v>45504</v>
+        <v>45535</v>
       </c>
       <c r="B26" s="4">
         <v>27</v>
@@ -1775,24 +1786,24 @@
         <v>21</v>
       </c>
       <c r="E26" s="4">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="F26" s="4">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="3">
-        <v>45473</v>
+        <v>45504</v>
       </c>
       <c r="B27" s="4">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C27" s="4">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D27" s="4">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E27" s="4">
         <v>4.2</v>
@@ -1803,7 +1814,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="3">
-        <v>45443</v>
+        <v>45473</v>
       </c>
       <c r="B28" s="4">
         <v>24</v>
@@ -1823,7 +1834,7 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="3">
-        <v>45412</v>
+        <v>45443</v>
       </c>
       <c r="B29" s="4">
         <v>24</v>
@@ -1843,27 +1854,27 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="3">
-        <v>45382</v>
+        <v>45412</v>
       </c>
       <c r="B30" s="4">
-        <v>20.5</v>
+        <v>24</v>
       </c>
       <c r="C30" s="4">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D30" s="4">
-        <v>16.5</v>
+        <v>19</v>
       </c>
       <c r="E30" s="4">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
       <c r="F30" s="4">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="3">
-        <v>45351</v>
+        <v>45382</v>
       </c>
       <c r="B31" s="4">
         <v>20.5</v>
@@ -1883,7 +1894,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="3">
-        <v>45322</v>
+        <v>45351</v>
       </c>
       <c r="B32" s="4">
         <v>20.5</v>
@@ -1903,27 +1914,27 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="3">
-        <v>45291</v>
+        <v>45322</v>
       </c>
       <c r="B33" s="4">
-        <v>17.5</v>
+        <v>20.5</v>
       </c>
       <c r="C33" s="4">
-        <v>26.4</v>
+        <v>32</v>
       </c>
       <c r="D33" s="4">
-        <v>13.7</v>
+        <v>16.5</v>
       </c>
       <c r="E33" s="4">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="F33" s="4">
-        <v>1.65</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="3">
-        <v>45260</v>
+        <v>45291</v>
       </c>
       <c r="B34" s="4">
         <v>17.5</v>
@@ -1935,18 +1946,18 @@
         <v>13.7</v>
       </c>
       <c r="E34" s="4">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="F34" s="4">
-        <v>1.55</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="3">
-        <v>45230</v>
+        <v>45260</v>
       </c>
       <c r="B35" s="4">
-        <v>17</v>
+        <v>17.5</v>
       </c>
       <c r="C35" s="4">
         <v>26.4</v>
@@ -1955,35 +1966,35 @@
         <v>13.7</v>
       </c>
       <c r="E35" s="4">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="F35" s="4">
-        <v>1.5</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3">
-        <v>45199</v>
+        <v>45230</v>
       </c>
       <c r="B36" s="4">
-        <v>15.3</v>
+        <v>17</v>
       </c>
       <c r="C36" s="4">
-        <v>23.8</v>
+        <v>26.4</v>
       </c>
       <c r="D36" s="4">
-        <v>12.4</v>
+        <v>13.7</v>
       </c>
       <c r="E36" s="4">
-        <v>2.73</v>
+        <v>3</v>
       </c>
       <c r="F36" s="4">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="3">
-        <v>45169</v>
+        <v>45199</v>
       </c>
       <c r="B37" s="4">
         <v>15.3</v>
@@ -2003,101 +2014,121 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="3">
-        <v>45138</v>
+        <v>45169</v>
       </c>
       <c r="B38" s="4">
         <v>15.3</v>
       </c>
       <c r="C38" s="4">
-        <v>24.4</v>
+        <v>23.8</v>
       </c>
       <c r="D38" s="4">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="E38" s="4">
-        <v>2.8</v>
+        <v>2.73</v>
       </c>
       <c r="F38" s="4">
-        <v>1.34</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="3">
-        <v>45107</v>
+        <v>45138</v>
       </c>
       <c r="B39" s="4">
-        <v>14.835</v>
+        <v>15.3</v>
       </c>
       <c r="C39" s="4">
-        <v>24.8</v>
+        <v>24.4</v>
       </c>
       <c r="D39" s="4">
-        <v>12.9</v>
+        <v>12.7</v>
       </c>
       <c r="E39" s="4">
-        <v>2.85</v>
+        <v>2.8</v>
       </c>
       <c r="F39" s="4">
-        <v>1.36</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="3">
-        <v>45077</v>
+        <v>45107</v>
       </c>
       <c r="B40" s="4">
-        <v>15.18</v>
+        <v>14.835</v>
       </c>
       <c r="C40" s="4">
-        <v>25.4</v>
+        <v>24.8</v>
       </c>
       <c r="D40" s="4">
-        <v>13.2</v>
+        <v>12.9</v>
       </c>
       <c r="E40" s="4">
-        <v>2.93</v>
+        <v>2.85</v>
       </c>
       <c r="F40" s="4">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="3">
-        <v>45046</v>
+        <v>45077</v>
       </c>
       <c r="B41" s="4">
-        <v>15.64</v>
+        <v>15.18</v>
       </c>
       <c r="C41" s="4">
-        <v>26.2</v>
+        <v>25.4</v>
       </c>
       <c r="D41" s="4">
-        <v>13.6</v>
+        <v>13.2</v>
       </c>
       <c r="E41" s="4">
-        <v>3.03</v>
+        <v>2.93</v>
       </c>
       <c r="F41" s="4">
-        <v>1.45</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="3">
+        <v>45046</v>
+      </c>
+      <c r="B42" s="4">
+        <v>15.64</v>
+      </c>
+      <c r="C42" s="4">
+        <v>26.2</v>
+      </c>
+      <c r="D42" s="4">
+        <v>13.6</v>
+      </c>
+      <c r="E42" s="4">
+        <v>3.03</v>
+      </c>
+      <c r="F42" s="4">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="5">
         <v>45016</v>
       </c>
-      <c r="B42" s="4">
+      <c r="B43" s="6">
         <v>18.975</v>
       </c>
-      <c r="C42" s="4">
+      <c r="C43" s="6">
         <v>32</v>
       </c>
-      <c r="D42" s="4">
+      <c r="D43" s="6">
         <v>16.5</v>
       </c>
-      <c r="E42" s="4">
+      <c r="E43" s="6">
         <v>3.75</v>
       </c>
-      <c r="F42" s="4">
+      <c r="F43" s="6">
         <v>1.81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update EDB prices for September 7
</commit_message>
<xml_diff>
--- a/edb_data/DRAM合约平均价格.xlsx
+++ b/edb_data/DRAM合约平均价格.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="24048" windowHeight="12300"/>
+    <workbookView windowWidth="27948" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="合约平均价_DRAM_DDR5(8Gb," sheetId="1" r:id="rId1"/>
@@ -710,19 +710,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -2113,22 +2107,22 @@
       </c>
     </row>
     <row r="43" spans="1:6">
-      <c r="A43" s="5">
+      <c r="A43" s="3">
         <v>45016</v>
       </c>
-      <c r="B43" s="6">
+      <c r="B43" s="4">
         <v>18.975</v>
       </c>
-      <c r="C43" s="6">
+      <c r="C43" s="4">
         <v>32</v>
       </c>
-      <c r="D43" s="6">
+      <c r="D43" s="4">
         <v>16.5</v>
       </c>
-      <c r="E43" s="6">
+      <c r="E43" s="4">
         <v>3.75</v>
       </c>
-      <c r="F43" s="6">
+      <c r="F43" s="4">
         <v>1.81</v>
       </c>
     </row>

</xml_diff>